<commit_message>
smoothed vib values and redid vas-vib with LMM
</commit_message>
<xml_diff>
--- a/our_data.xlsx
+++ b/our_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\Documents\GitHub\Databehandling_Med6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9DD4BFF-95A9-4563-B4F6-6C96F18054AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FFA5EB0-A01C-48D5-93FF-9F8C08C00A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20712" yWindow="972" windowWidth="26448" windowHeight="16320" tabRatio="500" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29304" yWindow="648" windowWidth="26448" windowHeight="16320" tabRatio="500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VAS" sheetId="1" r:id="rId1"/>
@@ -33,9 +33,6 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
@@ -252,7 +249,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -311,6 +308,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
@@ -493,11 +497,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -531,10 +536,14 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{ED72075D-43D1-439C-9895-31447684FEC5}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -32929,7 +32938,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:J342"/>
+  <dimension ref="A1:N342"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.95" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.44140625" customWidth="1"/>
@@ -32942,7 +32951,7 @@
     <col min="10" max="10" width="8.88671875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>43</v>
       </c>
@@ -32974,7 +32983,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -33006,7 +33015,7 @@
         <v>0.34992710611188299</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -33038,7 +33047,7 @@
         <v>-0.52489065916782396</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>1</v>
       </c>
@@ -33049,10 +33058,10 @@
         <v>88.957080000000005</v>
       </c>
       <c r="D4" s="3">
-        <v>30.00001</v>
+        <v>75.631615236907706</v>
       </c>
       <c r="E4" s="3">
-        <v>30.00001</v>
+        <v>71.160690224438895</v>
       </c>
       <c r="F4" s="3">
         <v>0</v>
@@ -33070,7 +33079,7 @@
         <v>1.2247448713915901</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>1</v>
       </c>
@@ -33080,11 +33089,11 @@
       <c r="C5" s="3">
         <v>91.816599999999994</v>
       </c>
-      <c r="D5" s="3">
-        <v>137.78579999999999</v>
-      </c>
-      <c r="E5" s="3">
-        <v>137.78579999999999</v>
+      <c r="D5" s="35">
+        <v>69.838313940149604</v>
+      </c>
+      <c r="E5" s="35">
+        <v>57.814338428927599</v>
       </c>
       <c r="F5" s="3">
         <v>0</v>
@@ -33101,8 +33110,10 @@
       <c r="J5" s="3">
         <v>-1.0497813183356499</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M5" s="34"/>
+      <c r="N5" s="34"/>
+    </row>
+    <row r="6" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2</v>
       </c>
@@ -33134,7 +33145,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2</v>
       </c>
@@ -33166,7 +33177,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2</v>
       </c>
@@ -33177,10 +33188,10 @@
         <v>90.656800000000004</v>
       </c>
       <c r="D8">
-        <v>30.00001</v>
+        <v>48.871773815461303</v>
       </c>
       <c r="E8">
-        <v>30.00001</v>
+        <v>53.600028503740603</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -33198,7 +33209,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2</v>
       </c>
@@ -33209,10 +33220,10 @@
         <v>91.036739999999995</v>
       </c>
       <c r="D9">
-        <v>30.00001</v>
+        <v>52.528617680798</v>
       </c>
       <c r="E9">
-        <v>30.000019999999999</v>
+        <v>78.403673416458801</v>
       </c>
       <c r="F9">
         <v>0.64472969999999996</v>
@@ -33230,7 +33241,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>3</v>
       </c>
@@ -33262,7 +33273,7 @@
         <v>1.4433756729740601</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>3</v>
       </c>
@@ -33294,7 +33305,7 @@
         <v>-0.28867513459481298</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>3</v>
       </c>
@@ -33305,10 +33316,10 @@
         <v>90.776780000000002</v>
       </c>
       <c r="D12" s="3">
-        <v>33.129719999999999</v>
+        <v>69.146842094763002</v>
       </c>
       <c r="E12" s="3">
-        <v>82.151439999999994</v>
+        <v>53.602109052369002</v>
       </c>
       <c r="F12" s="3">
         <v>0</v>
@@ -33325,8 +33336,10 @@
       <c r="J12" s="3">
         <v>-0.86602540378443904</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L12" s="33"/>
+      <c r="M12" s="33"/>
+    </row>
+    <row r="13" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>3</v>
       </c>
@@ -33337,10 +33350,10 @@
         <v>91.156720000000007</v>
       </c>
       <c r="D13" s="3">
-        <v>122.81359999999999</v>
+        <v>68.802924064837896</v>
       </c>
       <c r="E13" s="3">
-        <v>122.836</v>
+        <v>72.316895436408899</v>
       </c>
       <c r="F13" s="3">
         <v>0.80312450000000002</v>
@@ -33358,7 +33371,7 @@
         <v>-0.28867513459481298</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="27">
         <v>6</v>
       </c>
@@ -33390,7 +33403,7 @@
         <v>1.3228756555323</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>6</v>
       </c>
@@ -33422,7 +33435,7 @@
         <v>-0.94491118252306805</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>6</v>
       </c>
@@ -33433,10 +33446,10 @@
         <v>90.21687</v>
       </c>
       <c r="D16">
-        <v>99.344210000000004</v>
+        <v>76.190556059850294</v>
       </c>
       <c r="E16">
-        <v>63.910890000000002</v>
+        <v>68.230820822942604</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -33465,10 +33478,10 @@
         <v>90.89676</v>
       </c>
       <c r="D17">
-        <v>142.56200000000001</v>
+        <v>64.836995137157103</v>
       </c>
       <c r="E17">
-        <v>142.6456</v>
+        <v>81.602946284289203</v>
       </c>
       <c r="F17">
         <v>0.66206640000000005</v>
@@ -33561,10 +33574,10 @@
         <v>92.876429999999999</v>
       </c>
       <c r="D20" s="3">
-        <v>30.01333</v>
+        <v>60.326116558603402</v>
       </c>
       <c r="E20" s="3">
-        <v>30.01333</v>
+        <v>64.373301895261804</v>
       </c>
       <c r="F20" s="3">
         <v>0</v>
@@ -33593,10 +33606,10 @@
         <v>96.655789999999996</v>
       </c>
       <c r="D21" s="3">
-        <v>86.67107</v>
+        <v>86.545858927680797</v>
       </c>
       <c r="E21" s="3">
-        <v>103.20180000000001</v>
+        <v>79.291061271820396</v>
       </c>
       <c r="F21" s="3">
         <v>1</v>
@@ -33689,10 +33702,10 @@
         <v>102.25490000000001</v>
       </c>
       <c r="D24">
-        <v>30.000039999999998</v>
+        <v>52.681495935161998</v>
       </c>
       <c r="E24">
-        <v>75.00009</v>
+        <v>81.273257605984995</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -33721,10 +33734,10 @@
         <v>94.856089999999995</v>
       </c>
       <c r="D25">
-        <v>70.161680000000004</v>
+        <v>52.243764039900199</v>
       </c>
       <c r="E25">
-        <v>55.683109999999999</v>
+        <v>50.1080992518703</v>
       </c>
       <c r="F25">
         <v>1</v>
@@ -33817,10 +33830,10 @@
         <v>91.076729999999998</v>
       </c>
       <c r="D28" s="3">
-        <v>97.484899999999996</v>
+        <v>77.705092294264304</v>
       </c>
       <c r="E28" s="3">
-        <v>38.994109999999999</v>
+        <v>71.276398902743097</v>
       </c>
       <c r="F28" s="3">
         <v>0</v>
@@ -33849,10 +33862,10 @@
         <v>90.836770000000001</v>
       </c>
       <c r="D29" s="3">
-        <v>91.808909999999997</v>
+        <v>68.511969900249298</v>
       </c>
       <c r="E29" s="3">
-        <v>57.721899999999998</v>
+        <v>51.779723117206899</v>
       </c>
       <c r="F29" s="3">
         <v>0.36028640000000001</v>
@@ -33945,10 +33958,10 @@
         <v>90.496830000000003</v>
       </c>
       <c r="D32">
-        <v>36.798679999999997</v>
+        <v>75.458723665835393</v>
       </c>
       <c r="E32">
-        <v>74.342879999999994</v>
+        <v>67.413807306733105</v>
       </c>
       <c r="F32">
         <v>0</v>
@@ -33977,10 +33990,10 @@
         <v>91.156720000000007</v>
       </c>
       <c r="D33">
-        <v>30.00001</v>
+        <v>68.913383067331594</v>
       </c>
       <c r="E33">
-        <v>30.00001</v>
+        <v>55.712204987531102</v>
       </c>
       <c r="F33">
         <v>0</v>
@@ -34026,7 +34039,9 @@
       <c r="I34" s="3">
         <v>-0.5</v>
       </c>
-      <c r="J34" s="3"/>
+      <c r="J34" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="35" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="3">
@@ -34056,7 +34071,9 @@
       <c r="I35" s="3">
         <v>-0.5</v>
       </c>
-      <c r="J35" s="3"/>
+      <c r="J35" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="36" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
@@ -34069,10 +34086,10 @@
         <v>90.636799999999994</v>
       </c>
       <c r="D36" s="3">
-        <v>146.74039999999999</v>
+        <v>75.824719077306696</v>
       </c>
       <c r="E36" s="3">
-        <v>146.66390000000001</v>
+        <v>81.645339875311706</v>
       </c>
       <c r="F36" s="3">
         <v>0</v>
@@ -34086,7 +34103,9 @@
       <c r="I36" s="3">
         <v>-0.5</v>
       </c>
-      <c r="J36" s="3"/>
+      <c r="J36" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="37" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
@@ -34099,10 +34118,10 @@
         <v>91.356679999999997</v>
       </c>
       <c r="D37" s="3">
-        <v>66.054749999999999</v>
+        <v>87.992013915211899</v>
       </c>
       <c r="E37" s="3">
-        <v>103.1328</v>
+        <v>79.886956408977497</v>
       </c>
       <c r="F37" s="3">
         <v>0</v>
@@ -34116,7 +34135,9 @@
       <c r="I37" s="3">
         <v>-0.5</v>
       </c>
-      <c r="J37" s="3"/>
+      <c r="J37" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="38" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38">
@@ -34193,10 +34214,10 @@
         <v>89.578479999999999</v>
       </c>
       <c r="D40">
-        <v>57.863770000000002</v>
+        <v>63.784207639860099</v>
       </c>
       <c r="E40">
-        <v>57.854610000000001</v>
+        <v>64.008342080419496</v>
       </c>
       <c r="F40">
         <v>0</v>
@@ -34225,10 +34246,10 @@
         <v>90.985200000000006</v>
       </c>
       <c r="D41">
-        <v>30.00001</v>
+        <v>67.189837495590794</v>
       </c>
       <c r="E41">
-        <v>30.00001</v>
+        <v>63.254079929453198</v>
       </c>
       <c r="F41">
         <v>0</v>
@@ -34321,10 +34342,10 @@
         <v>106.39870000000001</v>
       </c>
       <c r="D44" s="3">
-        <v>64.507339999999999</v>
+        <v>45.744362062937</v>
       </c>
       <c r="E44" s="3">
-        <v>31.596990000000002</v>
+        <v>66.763422325174801</v>
       </c>
       <c r="F44" s="3">
         <v>0</v>
@@ -34353,10 +34374,10 @@
         <v>95.397450000000006</v>
       </c>
       <c r="D45" s="3">
-        <v>30</v>
+        <v>39.390092862129102</v>
       </c>
       <c r="E45" s="3">
-        <v>30</v>
+        <v>36.6344722513089</v>
       </c>
       <c r="F45" s="3">
         <v>0.95442159999999998</v>
@@ -34449,10 +34470,10 @@
         <v>97.740939999999995</v>
       </c>
       <c r="D48">
-        <v>61.295490000000001</v>
+        <v>48.357368656195398</v>
       </c>
       <c r="E48">
-        <v>104.8665</v>
+        <v>60.728186265270502</v>
       </c>
       <c r="F48">
         <v>0</v>
@@ -34481,10 +34502,10 @@
         <v>91.528459999999995</v>
       </c>
       <c r="D49">
-        <v>30</v>
+        <v>41.013634965034903</v>
       </c>
       <c r="E49">
-        <v>74.999979999999994</v>
+        <v>60.179631276223702</v>
       </c>
       <c r="F49">
         <v>1</v>
@@ -34577,10 +34598,10 @@
         <v>91.056730000000002</v>
       </c>
       <c r="D52" s="3">
-        <v>50.233330000000002</v>
+        <v>54.344690573565998</v>
       </c>
       <c r="E52" s="3">
-        <v>80.063670000000002</v>
+        <v>55.028385760598503</v>
       </c>
       <c r="F52" s="3">
         <v>0</v>
@@ -34609,10 +34630,10 @@
         <v>91.256699999999995</v>
       </c>
       <c r="D53" s="3">
-        <v>57.244570000000003</v>
+        <v>93.700114837905204</v>
       </c>
       <c r="E53" s="3">
-        <v>110.96639999999999</v>
+        <v>70.379248453865301</v>
       </c>
       <c r="F53" s="3">
         <v>0.81124419999999997</v>
@@ -34705,10 +34726,10 @@
         <v>91.656630000000007</v>
       </c>
       <c r="D56">
-        <v>118.72280000000001</v>
+        <v>90.844232643391507</v>
       </c>
       <c r="E56">
-        <v>119.74290000000001</v>
+        <v>90.486868279301703</v>
       </c>
       <c r="F56">
         <v>0</v>
@@ -34737,10 +34758,10 @@
         <v>90.89676</v>
       </c>
       <c r="D57">
-        <v>30.01886</v>
+        <v>61.5273018952618</v>
       </c>
       <c r="E57">
-        <v>30.01886</v>
+        <v>60.318408877805403</v>
       </c>
       <c r="F57">
         <v>1</v>
@@ -34833,10 +34854,10 @@
         <v>91.236699999999999</v>
       </c>
       <c r="D60" s="3">
-        <v>31.490469999999998</v>
+        <v>57.467885710723102</v>
       </c>
       <c r="E60" s="3">
-        <v>31.490950000000002</v>
+        <v>57.458658902743103</v>
       </c>
       <c r="F60" s="3">
         <v>0</v>
@@ -34865,10 +34886,10 @@
         <v>90.936750000000004</v>
       </c>
       <c r="D61" s="3">
-        <v>30.00001</v>
+        <v>65.336635885286697</v>
       </c>
       <c r="E61" s="3">
-        <v>30.00001</v>
+        <v>63.821912618453801</v>
       </c>
       <c r="F61" s="3">
         <v>0</v>
@@ -34961,10 +34982,10 @@
         <v>91.496660000000006</v>
       </c>
       <c r="D64">
-        <v>30.00001</v>
+        <v>30.891567306733101</v>
       </c>
       <c r="E64">
-        <v>75.000029999999995</v>
+        <v>76.984376608478797</v>
       </c>
       <c r="F64">
         <v>0</v>
@@ -34993,10 +35014,10 @@
         <v>92.036569999999998</v>
       </c>
       <c r="D65">
-        <v>30.23978</v>
+        <v>47.635911147132099</v>
       </c>
       <c r="E65">
-        <v>75.599429999999998</v>
+        <v>57.874344139650802</v>
       </c>
       <c r="F65">
         <v>0</v>

</xml_diff>